<commit_message>
Add chorus and achievement systems
</commit_message>
<xml_diff>
--- a/assets_cropped/Air Groove/manifest_edit.xlsx
+++ b/assets_cropped/Air Groove/manifest_edit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\TanukiProject\tanuki_app\assets_cropped\Air Groove\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D202F6-825D-4117-83CD-01A50F671F2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F236D9A-DF0B-4EB3-B75F-1F094221DB54}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="93">
   <si>
     <t>filename</t>
   </si>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t>idle_side-happy.gif</t>
-  </si>
-  <si>
-    <t>window_perch,observe_hold,bottle_feed_watch,shared_food_react,random</t>
   </si>
   <si>
     <t>idle_side-sad.gif</t>
@@ -284,27 +281,35 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_perch,relation_close,bottle_feed_watch,shared_food_react,random,activity_sleep_observing</t>
+    <t>activity_chorus_perform</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_perch,observe_hold,offer_timeout_route_a_step2,honey_guard_take,bottle_feed_watch,shared_food_react,random,activity_sleep_observing</t>
+    <t>window_walk,random,shared_food_approach,activity_sleep_join_approach,activity_chorus_approach</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_walk,random,activity_sleep_join_approach</t>
+    <t>window_walk,random,activity_sleep_join_approach,activity_chorus_approach</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_walk,random,shared_food_approach,activity_sleep_join_approach</t>
+    <t>window_perch,relation_close,bottle_feed_watch,shared_food_react,random,activity_sleep_observing,activity_chorus_observe</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_perch,care_companion,relation_close,bottle_feed_watch,shared_food_react,random,activity_sleep_join_settling</t>
+    <t>window_perch,observe_hold,offer_timeout_route_a_step2,honey_guard_take,bottle_feed_watch,shared_food_react,random,activity_sleep_observing,activity_chorus_observe</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>window_perch,relation_close,honey_guard_take,bottle_feed_watch,shared_food_react,random,activity_sleep_join_settling</t>
+    <t>window_perch,observe_hold,bottle_feed_watch,shared_food_react,random,activity_chorus_finish</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,relation_close,honey_guard_take,bottle_feed_watch,shared_food_react,random,activity_sleep_join_settling,activity_chorus_observe</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_companion,relation_close,bottle_feed_watch,shared_food_react,random,activity_sleep_join_settling,activity_chorus_observe</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -698,7 +703,7 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -726,7 +731,7 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -754,7 +759,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -768,7 +773,7 @@
         <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -810,7 +815,7 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -824,7 +829,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -838,7 +843,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -852,7 +857,7 @@
         <v>6</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -865,8 +870,8 @@
       <c r="B17" t="s">
         <v>6</v>
       </c>
-      <c r="C17" t="s">
-        <v>28</v>
+      <c r="C17" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -893,8 +898,8 @@
       <c r="B19" t="s">
         <v>13</v>
       </c>
-      <c r="C19" t="s">
-        <v>33</v>
+      <c r="C19" s="3" t="s">
+        <v>90</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -902,13 +907,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -916,13 +921,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
         <v>35</v>
-      </c>
-      <c r="B21" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" t="s">
-        <v>36</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -930,13 +935,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" t="s">
         <v>13</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -944,7 +949,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23" t="s">
         <v>10</v>
@@ -958,7 +963,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
@@ -972,7 +977,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
@@ -986,13 +991,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1000,13 +1005,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1014,13 +1019,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B28" t="s">
         <v>13</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1028,7 +1033,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
         <v>10</v>
@@ -1042,13 +1047,13 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B30" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1056,13 +1061,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
         <v>48</v>
-      </c>
-      <c r="B31" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" t="s">
-        <v>49</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1073,13 +1078,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
         <v>50</v>
-      </c>
-      <c r="B32" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>51</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1090,13 +1095,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" t="s">
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1104,13 +1109,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34" t="s">
         <v>13</v>
       </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1118,13 +1123,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B35" t="s">
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -1132,13 +1137,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s">
         <v>57</v>
-      </c>
-      <c r="B36" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" t="s">
-        <v>58</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1146,13 +1151,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" t="s">
         <v>13</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1160,13 +1165,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" t="s">
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1174,13 +1179,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
       </c>
       <c r="C39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1188,13 +1193,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B40" t="s">
         <v>13</v>
       </c>
       <c r="C40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1202,13 +1207,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B41" t="s">
         <v>10</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1216,13 +1221,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
         <v>64</v>
-      </c>
-      <c r="B42" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" t="s">
-        <v>65</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1230,13 +1235,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B43" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1277,18 +1282,18 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" t="s">
         <v>67</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>68</v>
-      </c>
-      <c r="H1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -1297,19 +1302,19 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>73</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>74</v>
-      </c>
-      <c r="H2" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>